<commit_message>
Add Cricbuzz Playwright automation
</commit_message>
<xml_diff>
--- a/daily_report_2026-09-08.xlsx
+++ b/daily_report_2026-09-08.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\g.c.periyasamy\pyautogui Demo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{29236188-6F9B-47EB-8961-2E04900E9660}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{872E3E8D-D1FC-4779-9D42-4B31C9EE8DC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="340" yWindow="3040" windowWidth="14400" windowHeight="7280" xr2:uid="{ECFA584F-4E4A-4A1B-835B-6E4EF171EB0C}"/>
+    <workbookView xWindow="340" yWindow="3040" windowWidth="14400" windowHeight="7280" xr2:uid="{EE3DD7DA-F986-4E99-82CE-1891CCC3E5D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
     <t>Comment</t>
   </si>
   <si>
-    <t>Chennai: 32C</t>
+    <t>Chennai: 30C</t>
   </si>
   <si>
     <t>Warm day; suitable with precautions</t>
@@ -425,7 +425,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1B0EE4E-097A-4CA6-AD48-B3A352F19654}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A8594B3-1071-4A03-AC48-934063098F32}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -445,7 +445,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
-        <v>46273.72383101852</v>
+        <v>46273.918587962966</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>

</xml_diff>